<commit_message>
Se agregaron nuevas restricciones de negocio al documento, todavía falta definir plan de acción para mitigar los riesgos
</commit_message>
<xml_diff>
--- a/Documentacion/RestriccionesNegocio.xlsx
+++ b/Documentacion/RestriccionesNegocio.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/F3F179366C32E272/Documentos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanp\FlorLogic\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEA21A6A-27AB-4D0D-B787-9D2B4AF3D774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67566E7F-6AEE-4443-9789-58C72E0CEB9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{49B2EC2E-3F64-4369-B5EE-BCFE592BC9C3}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{49B2EC2E-3F64-4369-B5EE-BCFE592BC9C3}"/>
   </bookViews>
   <sheets>
     <sheet name="RestriccionesNegocio" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
   <si>
     <t>Tipo</t>
   </si>
@@ -106,6 +106,24 @@
   </si>
   <si>
     <t>Tipo restricción negocio</t>
+  </si>
+  <si>
+    <t>El despliegue e instrucción del sistema no puede retrasar las actividades operativas por más de 7 días.</t>
+  </si>
+  <si>
+    <t>Después de la temporada alta se espera un tiempo dónde la carga de actividades se reduce, sin embargo esta etapa es corta.</t>
+  </si>
+  <si>
+    <t>Resistencia al cambio y curva de adopción de los supervisores de campo.</t>
+  </si>
+  <si>
+    <t>El personal que recolecta esta información puede estar muy arraigado a las prácticas previas al sistema, lograr una fácil adopción en el personal es crítico para el éxito del negocio.</t>
+  </si>
+  <si>
+    <t>Disponibilidad limitada en fechas previas a la implementación para pruebas y entregas previas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debido a la corta brecha de tiempo no se podría realizar pruebas de campo previas o dar retroalimentación continua a los desarrolladores. </t>
   </si>
 </sst>
 </file>
@@ -236,9 +254,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -276,7 +294,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -382,7 +400,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -524,7 +542,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -532,14 +550,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D97DF75-6389-4910-8EA4-F72D0BE21394}">
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.25"/>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="18" style="1" customWidth="1"/>
-    <col min="2" max="2" width="55.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="47.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="34.85546875" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="10.85546875" style="1"/>
+    <col min="2" max="2" width="55.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="47.88671875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="34.88671875" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -556,7 +574,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="76.5">
+    <row r="2" spans="1:4" ht="72">
       <c r="A2" s="9" t="s">
         <v>4</v>
       </c>
@@ -568,7 +586,7 @@
       </c>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" ht="45.75">
+    <row r="3" spans="1:4" ht="43.2">
       <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
@@ -580,7 +598,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" ht="76.5">
+    <row r="4" spans="1:4" ht="72">
       <c r="A4" s="9" t="s">
         <v>10</v>
       </c>
@@ -592,7 +610,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:4" ht="91.5">
+    <row r="5" spans="1:4" ht="86.4">
       <c r="A5" s="9" t="s">
         <v>13</v>
       </c>
@@ -604,7 +622,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" ht="45.75">
+    <row r="6" spans="1:4" ht="43.2">
       <c r="A6" s="9" t="s">
         <v>7</v>
       </c>
@@ -616,7 +634,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" ht="60.75">
+    <row r="7" spans="1:4" ht="43.2">
       <c r="A7" s="9" t="s">
         <v>18</v>
       </c>
@@ -628,29 +646,53 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" ht="15">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="3"/>
-    </row>
-    <row r="9" spans="1:4" ht="15">
-      <c r="A9" s="9"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
+    <row r="8" spans="1:4" ht="43.2">
+      <c r="A8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" ht="57.6">
+      <c r="A9" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:4" ht="43.2">
+      <c r="A10" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="3"/>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -661,7 +703,7 @@
           <x14:formula1>
             <xm:f>Valores!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A9</xm:sqref>
+          <xm:sqref>A2:A10</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -672,7 +714,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAF3187D-6537-41A0-BC18-FEE60642C528}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
@@ -710,6 +752,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010013DED8002B981F47A2AB219162B18A45" ma:contentTypeVersion="3" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="11c75646286b434d6b62b79d62284a00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="77a89e33-5ee6-4ee5-94b3-3d8acedffa3b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b189093bc8542a5f2a6028f197033518" ns2:_="">
     <xsd:import namespace="77a89e33-5ee6-4ee5-94b3-3d8acedffa3b"/>
@@ -847,31 +904,39 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FE361FB-0854-48C1-92D7-A45A031C082E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAA0016E-02AD-40A7-B138-AC3800F21AD5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D600589F-502F-4268-B28C-05E55A079148}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D600589F-502F-4268-B28C-05E55A079148}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAA0016E-02AD-40A7-B138-AC3800F21AD5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FE361FB-0854-48C1-92D7-A45A031C082E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="77a89e33-5ee6-4ee5-94b3-3d8acedffa3b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>